<commit_message>
+ DATA REVERIFICATION CHANGE
</commit_message>
<xml_diff>
--- a/Nubank_Case_Performer/Data/Temp/Relatorio_Vendas_AGATHON TRADING.xlsx
+++ b/Nubank_Case_Performer/Data/Temp/Relatorio_Vendas_AGATHON TRADING.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinic\Documents\UiPath\Nubank_Case_Performer\Data\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEDA503F-233E-4028-8F1A-9B5E353E53ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB2F5985-D841-465F-9B86-804BD30E14F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2160" yWindow="2160" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="{ID_VENDOR}" sheetId="1" r:id="rId1"/>
@@ -86,7 +86,7 @@
     <t>FR065748</t>
   </si>
   <si>
-    <t>29/04/2026</t>
+    <t>05/05/2026</t>
   </si>
   <si>
     <t>AGATHON TRADING</t>
@@ -113,7 +113,7 @@
     <t>145432 / Concierge Services</t>
   </si>
   <si>
-    <t>Please, GENERATE INVOICES by 04/05/2026</t>
+    <t>Please, GENERATE INVOICES by 10/05/2026</t>
   </si>
 </sst>
 </file>
@@ -1449,14 +1449,14 @@
       </c>
       <c r="C18" s="44"/>
       <c r="D18" s="45">
-        <v>145948.24</v>
+        <v>143270.31</v>
       </c>
       <c r="E18" s="46">
         <v>7</v>
       </c>
       <c r="F18" s="44"/>
       <c r="G18" s="45">
-        <v>1021637.68</v>
+        <v>1002892.14</v>
       </c>
       <c r="H18" s="10"/>
       <c r="I18" s="1"/>
@@ -1485,14 +1485,14 @@
       </c>
       <c r="C19" s="44"/>
       <c r="D19" s="47">
-        <v>192368.32</v>
+        <v>190144.61</v>
       </c>
       <c r="E19" s="46">
         <v>10</v>
       </c>
       <c r="F19" s="44"/>
       <c r="G19" s="45">
-        <v>1923683.15</v>
+        <v>1901446.13</v>
       </c>
       <c r="H19" s="18"/>
       <c r="I19" s="1"/>
@@ -1521,14 +1521,14 @@
       </c>
       <c r="C20" s="44"/>
       <c r="D20" s="47">
-        <v>97586.48</v>
+        <v>95795.92</v>
       </c>
       <c r="E20" s="46">
         <v>9</v>
       </c>
       <c r="F20" s="44"/>
       <c r="G20" s="45">
-        <v>878278.36</v>
+        <v>862163.26</v>
       </c>
       <c r="H20" s="10"/>
       <c r="I20" s="1"/>
@@ -1766,7 +1766,7 @@
       <c r="F27" s="56"/>
       <c r="G27" s="57">
         <f>SUM(G18:G25)</f>
-        <v>3823599.19</v>
+        <v>3766501.5300000003</v>
       </c>
       <c r="H27" s="20"/>
       <c r="I27" s="1"/>
@@ -1792,7 +1792,7 @@
       <c r="A28" s="19"/>
       <c r="B28" s="58">
         <f>G31</f>
-        <v>3613301.2335000001</v>
+        <v>3559343.9490000005</v>
       </c>
       <c r="C28" s="54"/>
       <c r="D28" s="54"/>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="F28" s="56"/>
       <c r="G28" s="57">
-        <v>382359.92</v>
+        <v>376650.15</v>
       </c>
       <c r="H28" s="20"/>
       <c r="I28" s="1"/>
@@ -1866,7 +1866,7 @@
       <c r="F30" s="56"/>
       <c r="G30" s="57">
         <f>(G27-G28)*G29</f>
-        <v>172061.96350000001</v>
+        <v>169492.56900000002</v>
       </c>
       <c r="H30" s="20"/>
       <c r="I30" s="1"/>
@@ -1899,7 +1899,7 @@
       <c r="F31" s="56"/>
       <c r="G31" s="57">
         <f>G27-G28+G30</f>
-        <v>3613301.2335000001</v>
+        <v>3559343.9490000005</v>
       </c>
       <c r="H31" s="20"/>
       <c r="I31" s="1"/>

</xml_diff>